<commit_message>
Complete Sprint 3 - Screening and Peer Analytics
</commit_message>
<xml_diff>
--- a/data/raw/documents.xlsx
+++ b/data/raw/documents.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Documents" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Documents'!$A$2:$D$2</definedName>
@@ -978,11 +978,7 @@
       <c r="C28" s="5" t="n">
         <v>2015</v>
       </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -996,11 +992,7 @@
       <c r="C29" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
@@ -1014,11 +1006,7 @@
       <c r="C30" s="5" t="n">
         <v>2013</v>
       </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -1032,11 +1020,7 @@
       <c r="C31" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
@@ -1050,11 +1034,7 @@
       <c r="C32" s="5" t="n">
         <v>2011</v>
       </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -1068,11 +1048,7 @@
       <c r="C33" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
@@ -1086,11 +1062,7 @@
       <c r="C34" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -1338,7 +1310,9 @@
       <c r="C48" s="5" t="n">
         <v>2011</v>
       </c>
-      <c r="D48" s="6" t="n"/>
+      <c r="D48" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -1352,7 +1326,9 @@
       <c r="C49" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D49" s="4" t="n"/>
+      <c r="D49" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n">
@@ -1366,7 +1342,9 @@
       <c r="C50" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D50" s="6" t="n"/>
+      <c r="D50" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
@@ -1506,11 +1484,7 @@
       <c r="C58" s="5" t="n">
         <v>2017</v>
       </c>
-      <c r="D58" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D58" s="6" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
@@ -1524,11 +1498,7 @@
       <c r="C59" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n">
@@ -1542,11 +1512,7 @@
       <c r="C60" s="5" t="n">
         <v>2015</v>
       </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D60" s="6" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n">
@@ -1560,11 +1526,7 @@
       <c r="C61" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="D61" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n">
@@ -1578,11 +1540,7 @@
       <c r="C62" s="5" t="n">
         <v>2013</v>
       </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D62" s="6" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
@@ -1596,11 +1554,7 @@
       <c r="C63" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n">
@@ -1614,11 +1568,7 @@
       <c r="C64" s="5" t="n">
         <v>2011</v>
       </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D64" s="6" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
@@ -1632,11 +1582,7 @@
       <c r="C65" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
@@ -1650,11 +1596,7 @@
       <c r="C66" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D66" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D66" s="6" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
@@ -1758,11 +1700,7 @@
       <c r="C72" s="5" t="n">
         <v>2019</v>
       </c>
-      <c r="D72" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D72" s="6" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n">
@@ -1776,11 +1714,7 @@
       <c r="C73" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D73" s="4" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="n">
@@ -1794,11 +1728,7 @@
       <c r="C74" s="5" t="n">
         <v>2017</v>
       </c>
-      <c r="D74" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D74" s="6" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n">
@@ -1830,11 +1760,7 @@
       <c r="C76" s="5" t="n">
         <v>2015</v>
       </c>
-      <c r="D76" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D76" s="6" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n">
@@ -1848,11 +1774,7 @@
       <c r="C77" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D77" s="4" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="n">
@@ -1866,11 +1788,7 @@
       <c r="C78" s="5" t="n">
         <v>2013</v>
       </c>
-      <c r="D78" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D78" s="6" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n">
@@ -1884,11 +1802,7 @@
       <c r="C79" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="D79" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D79" s="4" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n">
@@ -1920,11 +1834,7 @@
       <c r="C81" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D81" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D81" s="4" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
@@ -1938,11 +1848,7 @@
       <c r="C82" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D82" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D82" s="6" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n">
@@ -2118,11 +2024,7 @@
       <c r="C92" s="5" t="n">
         <v>2015</v>
       </c>
-      <c r="D92" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D92" s="6" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="n">
@@ -2136,11 +2038,7 @@
       <c r="C93" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="D93" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D93" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="5" t="n">
@@ -2154,11 +2052,7 @@
       <c r="C94" s="5" t="n">
         <v>2013</v>
       </c>
-      <c r="D94" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D94" s="6" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n">
@@ -2190,11 +2084,7 @@
       <c r="C96" s="5" t="n">
         <v>2011</v>
       </c>
-      <c r="D96" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D96" s="6" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n">
@@ -2208,11 +2098,7 @@
       <c r="C97" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D97" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D97" s="4" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="n">
@@ -2226,11 +2112,7 @@
       <c r="C98" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D98" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D98" s="6" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="n">
@@ -2424,11 +2306,7 @@
       <c r="C109" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="D109" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D109" s="4" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="5" t="n">
@@ -2442,11 +2320,7 @@
       <c r="C110" s="5" t="n">
         <v>2013</v>
       </c>
-      <c r="D110" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D110" s="6" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="3" t="n">
@@ -2460,11 +2334,7 @@
       <c r="C111" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="D111" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D111" s="4" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="n">
@@ -2496,11 +2366,7 @@
       <c r="C113" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D113" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="5" t="n">
@@ -2514,11 +2380,7 @@
       <c r="C114" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D114" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D114" s="6" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="3" t="n">
@@ -2622,11 +2484,7 @@
       <c r="C120" s="5" t="n">
         <v>2019</v>
       </c>
-      <c r="D120" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D120" s="6" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="3" t="n">
@@ -2694,11 +2552,7 @@
       <c r="C124" s="5" t="n">
         <v>2015</v>
       </c>
-      <c r="D124" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D124" s="6" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="3" t="n">
@@ -2784,11 +2638,7 @@
       <c r="C129" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D129" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D129" s="4" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="5" t="n">
@@ -2802,11 +2652,7 @@
       <c r="C130" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D130" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D130" s="6" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="3" t="n">
@@ -3018,11 +2864,7 @@
       <c r="C142" s="5" t="n">
         <v>2013</v>
       </c>
-      <c r="D142" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D142" s="6" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="3" t="n">
@@ -3036,11 +2878,7 @@
       <c r="C143" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="D143" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D143" s="4" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="5" t="n">
@@ -3072,11 +2910,7 @@
       <c r="C145" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D145" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D145" s="4" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="n">
@@ -3090,11 +2924,7 @@
       <c r="C146" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D146" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D146" s="6" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="3" t="n">
@@ -3216,11 +3046,7 @@
       <c r="C153" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="D153" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D153" s="4" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="5" t="n">
@@ -3234,11 +3060,7 @@
       <c r="C154" s="5" t="n">
         <v>2017</v>
       </c>
-      <c r="D154" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D154" s="6" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="3" t="n">
@@ -3252,11 +3074,7 @@
       <c r="C155" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="D155" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D155" s="4" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="5" t="n">
@@ -3270,11 +3088,7 @@
       <c r="C156" s="5" t="n">
         <v>2015</v>
       </c>
-      <c r="D156" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D156" s="6" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="3" t="n">
@@ -3288,11 +3102,7 @@
       <c r="C157" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="D157" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D157" s="4" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="5" t="n">
@@ -3306,11 +3116,7 @@
       <c r="C158" s="5" t="n">
         <v>2013</v>
       </c>
-      <c r="D158" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D158" s="6" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="3" t="n">
@@ -3324,11 +3130,7 @@
       <c r="C159" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="D159" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D159" s="4" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="5" t="n">
@@ -3342,11 +3144,7 @@
       <c r="C160" s="5" t="n">
         <v>2011</v>
       </c>
-      <c r="D160" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D160" s="6" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="3" t="n">
@@ -3360,11 +3158,7 @@
       <c r="C161" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D161" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D161" s="4" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="5" t="n">
@@ -3378,11 +3172,7 @@
       <c r="C162" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D162" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D162" s="6" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="3" t="n">
@@ -3648,11 +3438,7 @@
       <c r="C177" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D177" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D177" s="4" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="5" t="n">
@@ -3666,11 +3452,7 @@
       <c r="C178" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D178" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D178" s="6" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="3" t="n">
@@ -3864,11 +3646,7 @@
       <c r="C189" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="D189" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D189" s="4" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="5" t="n">
@@ -3936,11 +3714,7 @@
       <c r="C193" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D193" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D193" s="4" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="5" t="n">
@@ -3954,11 +3728,7 @@
       <c r="C194" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D194" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D194" s="6" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="3" t="n">
@@ -4224,11 +3994,7 @@
       <c r="C209" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D209" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D209" s="4" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="5" t="n">
@@ -4242,11 +4008,7 @@
       <c r="C210" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D210" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D210" s="6" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="3" t="n">
@@ -4512,11 +4274,7 @@
       <c r="C225" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D225" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D225" s="4" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="5" t="n">
@@ -4530,11 +4288,7 @@
       <c r="C226" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D226" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D226" s="6" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="3" t="n">
@@ -4800,11 +4554,7 @@
       <c r="C241" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D241" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D241" s="4" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="5" t="n">
@@ -4818,11 +4568,7 @@
       <c r="C242" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D242" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D242" s="6" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="3" t="n">
@@ -5088,7 +4834,9 @@
       <c r="C257" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D257" s="4" t="n"/>
+      <c r="D257" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="5" t="n">
@@ -5102,7 +4850,9 @@
       <c r="C258" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D258" s="6" t="n"/>
+      <c r="D258" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="3" t="n">
@@ -5152,7 +4902,9 @@
       <c r="C261" s="3" t="n">
         <v>2022</v>
       </c>
-      <c r="D261" s="4" t="n"/>
+      <c r="D261" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="5" t="n">
@@ -5202,7 +4954,9 @@
       <c r="C264" s="5" t="n">
         <v>2019</v>
       </c>
-      <c r="D264" s="6" t="n"/>
+      <c r="D264" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="3" t="n">
@@ -5270,7 +5024,9 @@
       <c r="C268" s="5" t="n">
         <v>2015</v>
       </c>
-      <c r="D268" s="6" t="n"/>
+      <c r="D268" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="3" t="n">
@@ -5320,7 +5076,9 @@
       <c r="C271" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="D271" s="4" t="n"/>
+      <c r="D271" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="5" t="n">
@@ -5334,7 +5092,9 @@
       <c r="C272" s="5" t="n">
         <v>2011</v>
       </c>
-      <c r="D272" s="6" t="n"/>
+      <c r="D272" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="3" t="n">
@@ -5348,7 +5108,9 @@
       <c r="C273" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D273" s="4" t="n"/>
+      <c r="D273" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="5" t="n">
@@ -5362,7 +5124,9 @@
       <c r="C274" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D274" s="6" t="n"/>
+      <c r="D274" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="3" t="n">
@@ -5430,7 +5194,9 @@
       <c r="C278" s="5" t="n">
         <v>2021</v>
       </c>
-      <c r="D278" s="6" t="n"/>
+      <c r="D278" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="3" t="n">
@@ -5480,7 +5246,9 @@
       <c r="C281" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="D281" s="4" t="n"/>
+      <c r="D281" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="5" t="n">
@@ -5602,7 +5370,9 @@
       <c r="C288" s="5" t="n">
         <v>2011</v>
       </c>
-      <c r="D288" s="6" t="n"/>
+      <c r="D288" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="3" t="n">
@@ -5616,7 +5386,9 @@
       <c r="C289" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D289" s="4" t="n"/>
+      <c r="D289" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="5" t="n">
@@ -5630,7 +5402,9 @@
       <c r="C290" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D290" s="6" t="n"/>
+      <c r="D290" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="3" t="n">
@@ -5806,7 +5580,9 @@
       <c r="C300" s="5" t="n">
         <v>2015</v>
       </c>
-      <c r="D300" s="6" t="n"/>
+      <c r="D300" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="3" t="n">
@@ -5820,7 +5596,9 @@
       <c r="C301" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="D301" s="4" t="n"/>
+      <c r="D301" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="5" t="n">
@@ -5834,7 +5612,9 @@
       <c r="C302" s="5" t="n">
         <v>2013</v>
       </c>
-      <c r="D302" s="6" t="n"/>
+      <c r="D302" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="3" t="n">
@@ -5848,7 +5628,9 @@
       <c r="C303" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="D303" s="4" t="n"/>
+      <c r="D303" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="5" t="n">
@@ -5862,7 +5644,9 @@
       <c r="C304" s="5" t="n">
         <v>2011</v>
       </c>
-      <c r="D304" s="6" t="n"/>
+      <c r="D304" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="3" t="n">
@@ -5876,7 +5660,9 @@
       <c r="C305" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D305" s="4" t="n"/>
+      <c r="D305" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="5" t="n">
@@ -5890,7 +5676,9 @@
       <c r="C306" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D306" s="6" t="n"/>
+      <c r="D306" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="3" t="n">
@@ -5994,7 +5782,9 @@
       <c r="C312" s="5" t="n">
         <v>2019</v>
       </c>
-      <c r="D312" s="6" t="n"/>
+      <c r="D312" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="3" t="n">
@@ -6008,7 +5798,9 @@
       <c r="C313" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="D313" s="4" t="n"/>
+      <c r="D313" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="5" t="n">
@@ -6022,7 +5814,9 @@
       <c r="C314" s="5" t="n">
         <v>2017</v>
       </c>
-      <c r="D314" s="6" t="n"/>
+      <c r="D314" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="3" t="n">
@@ -6072,7 +5866,9 @@
       <c r="C317" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="D317" s="4" t="n"/>
+      <c r="D317" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="5" t="n">
@@ -6086,7 +5882,9 @@
       <c r="C318" s="5" t="n">
         <v>2013</v>
       </c>
-      <c r="D318" s="6" t="n"/>
+      <c r="D318" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="3" t="n">
@@ -6100,7 +5898,9 @@
       <c r="C319" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="D319" s="4" t="n"/>
+      <c r="D319" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="5" t="n">
@@ -6114,7 +5914,9 @@
       <c r="C320" s="5" t="n">
         <v>2011</v>
       </c>
-      <c r="D320" s="6" t="n"/>
+      <c r="D320" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="3" t="n">
@@ -6128,7 +5930,9 @@
       <c r="C321" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D321" s="4" t="n"/>
+      <c r="D321" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="5" t="n">
@@ -6142,7 +5946,9 @@
       <c r="C322" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D322" s="6" t="n"/>
+      <c r="D322" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="3" t="n">
@@ -6192,7 +5998,9 @@
       <c r="C325" s="3" t="n">
         <v>2022</v>
       </c>
-      <c r="D325" s="4" t="n"/>
+      <c r="D325" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="5" t="n">
@@ -6242,7 +6050,9 @@
       <c r="C328" s="5" t="n">
         <v>2019</v>
       </c>
-      <c r="D328" s="6" t="n"/>
+      <c r="D328" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="3" t="n">
@@ -6292,7 +6102,9 @@
       <c r="C331" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="D331" s="4" t="n"/>
+      <c r="D331" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="5" t="n">
@@ -6306,7 +6118,9 @@
       <c r="C332" s="5" t="n">
         <v>2015</v>
       </c>
-      <c r="D332" s="6" t="n"/>
+      <c r="D332" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="3" t="n">
@@ -6392,7 +6206,9 @@
       <c r="C337" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D337" s="4" t="n"/>
+      <c r="D337" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="5" t="n">
@@ -6406,7 +6222,9 @@
       <c r="C338" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D338" s="6" t="n"/>
+      <c r="D338" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="3" t="n">
@@ -6672,11 +6490,7 @@
       <c r="C353" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D353" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D353" s="4" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="5" t="n">
@@ -6690,11 +6504,7 @@
       <c r="C354" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D354" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D354" s="6" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="3" t="n">
@@ -6960,11 +6770,7 @@
       <c r="C369" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D369" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D369" s="4" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="5" t="n">
@@ -6978,11 +6784,7 @@
       <c r="C370" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D370" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D370" s="6" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="3" t="n">
@@ -7158,11 +6960,7 @@
       <c r="C380" s="5" t="n">
         <v>2015</v>
       </c>
-      <c r="D380" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D380" s="6" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="3" t="n">
@@ -7248,11 +7046,7 @@
       <c r="C385" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D385" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D385" s="4" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="5" t="n">
@@ -7266,11 +7060,7 @@
       <c r="C386" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D386" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D386" s="6" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="3" t="n">
@@ -7536,11 +7326,7 @@
       <c r="C401" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D401" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D401" s="4" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="5" t="n">
@@ -7554,11 +7340,7 @@
       <c r="C402" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D402" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D402" s="6" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="3" t="n">
@@ -7824,11 +7606,7 @@
       <c r="C417" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D417" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D417" s="4" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="5" t="n">
@@ -8112,11 +7890,7 @@
       <c r="C433" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D433" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D433" s="4" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="5" t="n">
@@ -8130,11 +7904,7 @@
       <c r="C434" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D434" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D434" s="6" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="3" t="n">
@@ -8256,7 +8026,9 @@
       <c r="C441" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="D441" s="4" t="n"/>
+      <c r="D441" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="442">
       <c r="A442" s="5" t="n">
@@ -8270,7 +8042,9 @@
       <c r="C442" s="5" t="n">
         <v>2017</v>
       </c>
-      <c r="D442" s="6" t="n"/>
+      <c r="D442" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="443">
       <c r="A443" s="3" t="n">
@@ -8392,11 +8166,7 @@
       <c r="C449" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D449" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D449" s="4" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="5" t="n">
@@ -8410,11 +8180,7 @@
       <c r="C450" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D450" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D450" s="6" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="3" t="n">
@@ -8572,11 +8338,7 @@
       <c r="C459" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="D459" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D459" s="4" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="5" t="n">
@@ -8590,11 +8352,7 @@
       <c r="C460" s="5" t="n">
         <v>2015</v>
       </c>
-      <c r="D460" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D460" s="6" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="3" t="n">
@@ -8608,11 +8366,7 @@
       <c r="C461" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="D461" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D461" s="4" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="5" t="n">
@@ -8626,11 +8380,7 @@
       <c r="C462" s="5" t="n">
         <v>2013</v>
       </c>
-      <c r="D462" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D462" s="6" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="3" t="n">
@@ -8644,11 +8394,7 @@
       <c r="C463" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="D463" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D463" s="4" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="5" t="n">
@@ -8662,11 +8408,7 @@
       <c r="C464" s="5" t="n">
         <v>2011</v>
       </c>
-      <c r="D464" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D464" s="6" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="3" t="n">
@@ -8680,11 +8422,7 @@
       <c r="C465" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D465" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D465" s="4" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="5" t="n">
@@ -8698,11 +8436,7 @@
       <c r="C466" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D466" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D466" s="6" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="3" t="n">
@@ -8950,11 +8684,7 @@
       <c r="C480" s="5" t="n">
         <v>2011</v>
       </c>
-      <c r="D480" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D480" s="6" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="3" t="n">
@@ -8968,11 +8698,7 @@
       <c r="C481" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D481" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D481" s="4" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="5" t="n">
@@ -8986,11 +8712,7 @@
       <c r="C482" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D482" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D482" s="6" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="3" t="n">
@@ -9094,7 +8816,9 @@
       <c r="C488" s="5" t="n">
         <v>2019</v>
       </c>
-      <c r="D488" s="6" t="n"/>
+      <c r="D488" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="489">
       <c r="A489" s="3" t="n">
@@ -9252,11 +8976,7 @@
       <c r="C497" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D497" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D497" s="4" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="5" t="n">
@@ -9270,11 +8990,7 @@
       <c r="C498" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D498" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D498" s="6" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="3" t="n">
@@ -9540,11 +9256,7 @@
       <c r="C513" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D513" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D513" s="4" t="n"/>
     </row>
     <row r="514">
       <c r="A514" s="5" t="n">
@@ -9558,11 +9270,7 @@
       <c r="C514" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D514" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D514" s="6" t="n"/>
     </row>
     <row r="515">
       <c r="A515" s="3" t="n">
@@ -9828,11 +9536,7 @@
       <c r="C529" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D529" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D529" s="4" t="n"/>
     </row>
     <row r="530">
       <c r="A530" s="5" t="n">
@@ -9846,11 +9550,7 @@
       <c r="C530" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D530" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D530" s="6" t="n"/>
     </row>
     <row r="531">
       <c r="A531" s="3" t="n">
@@ -10116,11 +9816,7 @@
       <c r="C545" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="D545" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D545" s="4" t="n"/>
     </row>
     <row r="546">
       <c r="A546" s="5" t="n">
@@ -10134,11 +9830,7 @@
       <c r="C546" s="5" t="n">
         <v>2009</v>
       </c>
-      <c r="D546" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D546" s="6" t="n"/>
     </row>
     <row r="547">
       <c r="A547" s="3" t="n">
@@ -10386,7 +10078,9 @@
       <c r="C560" s="5" t="n">
         <v>2011</v>
       </c>
-      <c r="D560" s="6" t="n"/>
+      <c r="D560" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="561">
       <c r="A561" s="3" t="n">
@@ -10436,11 +10130,7 @@
       <c r="C563" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D563" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D563" s="4" t="n"/>
     </row>
     <row r="564">
       <c r="A564" s="5" t="n">
@@ -10670,11 +10360,7 @@
       <c r="C576" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D576" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D576" s="6" t="n"/>
     </row>
     <row r="577">
       <c r="A577" s="3" t="n">
@@ -10688,11 +10374,7 @@
       <c r="C577" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D577" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D577" s="4" t="n"/>
     </row>
     <row r="578">
       <c r="A578" s="5" t="n">
@@ -10940,11 +10622,7 @@
       <c r="C591" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D591" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D591" s="4" t="n"/>
     </row>
     <row r="592">
       <c r="A592" s="5" t="n">
@@ -10958,11 +10636,7 @@
       <c r="C592" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D592" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D592" s="6" t="n"/>
     </row>
     <row r="593">
       <c r="A593" s="3" t="n">
@@ -10976,11 +10650,7 @@
       <c r="C593" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D593" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D593" s="4" t="n"/>
     </row>
     <row r="594">
       <c r="A594" s="5" t="n">
@@ -11192,11 +10862,7 @@
       <c r="C605" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D605" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D605" s="4" t="n"/>
     </row>
     <row r="606">
       <c r="A606" s="5" t="n">
@@ -11228,11 +10894,7 @@
       <c r="C607" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D607" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D607" s="4" t="n"/>
     </row>
     <row r="608">
       <c r="A608" s="5" t="n">
@@ -11246,11 +10908,7 @@
       <c r="C608" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D608" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D608" s="6" t="n"/>
     </row>
     <row r="609">
       <c r="A609" s="3" t="n">
@@ -11264,11 +10922,7 @@
       <c r="C609" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D609" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D609" s="4" t="n"/>
     </row>
     <row r="610">
       <c r="A610" s="5" t="n">
@@ -11498,11 +11152,7 @@
       <c r="C622" s="5" t="n">
         <v>2012</v>
       </c>
-      <c r="D622" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D622" s="6" t="n"/>
     </row>
     <row r="623">
       <c r="A623" s="3" t="n">
@@ -11516,11 +11166,7 @@
       <c r="C623" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D623" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D623" s="4" t="n"/>
     </row>
     <row r="624">
       <c r="A624" s="5" t="n">
@@ -11534,11 +11180,7 @@
       <c r="C624" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D624" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D624" s="6" t="n"/>
     </row>
     <row r="625">
       <c r="A625" s="3" t="n">
@@ -11552,11 +11194,7 @@
       <c r="C625" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D625" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D625" s="4" t="n"/>
     </row>
     <row r="626">
       <c r="A626" s="5" t="n">
@@ -11570,11 +11208,7 @@
       <c r="C626" s="5" t="n">
         <v>2008</v>
       </c>
-      <c r="D626" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D626" s="6" t="n"/>
     </row>
     <row r="627">
       <c r="A627" s="3" t="n">
@@ -11858,11 +11492,7 @@
       <c r="C642" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D642" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D642" s="6" t="n"/>
     </row>
     <row r="643">
       <c r="A643" s="3" t="n">
@@ -11876,11 +11506,7 @@
       <c r="C643" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D643" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D643" s="4" t="n"/>
     </row>
     <row r="644">
       <c r="A644" s="5" t="n">
@@ -12146,11 +11772,7 @@
       <c r="C658" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D658" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D658" s="6" t="n"/>
     </row>
     <row r="659">
       <c r="A659" s="3" t="n">
@@ -12164,11 +11786,7 @@
       <c r="C659" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D659" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D659" s="4" t="n"/>
     </row>
     <row r="660">
       <c r="A660" s="5" t="n">
@@ -12434,11 +12052,7 @@
       <c r="C674" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D674" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D674" s="6" t="n"/>
     </row>
     <row r="675">
       <c r="A675" s="3" t="n">
@@ -12452,11 +12066,7 @@
       <c r="C675" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D675" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D675" s="4" t="n"/>
     </row>
     <row r="676">
       <c r="A676" s="5" t="n">
@@ -12740,11 +12350,7 @@
       <c r="C691" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D691" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D691" s="4" t="n"/>
     </row>
     <row r="692">
       <c r="A692" s="5" t="n">
@@ -13028,11 +12634,7 @@
       <c r="C707" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D707" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D707" s="4" t="n"/>
     </row>
     <row r="708">
       <c r="A708" s="5" t="n">
@@ -13280,11 +12882,7 @@
       <c r="C721" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D721" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D721" s="4" t="n"/>
     </row>
     <row r="722">
       <c r="A722" s="5" t="n">
@@ -13298,11 +12896,7 @@
       <c r="C722" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D722" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D722" s="6" t="n"/>
     </row>
     <row r="723">
       <c r="A723" s="3" t="n">
@@ -13316,11 +12910,7 @@
       <c r="C723" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D723" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D723" s="4" t="n"/>
     </row>
     <row r="724">
       <c r="A724" s="5" t="n">
@@ -13496,11 +13086,7 @@
       <c r="C733" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="D733" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D733" s="4" t="n"/>
     </row>
     <row r="734">
       <c r="A734" s="5" t="n">
@@ -13514,11 +13100,7 @@
       <c r="C734" s="5" t="n">
         <v>2014</v>
       </c>
-      <c r="D734" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D734" s="6" t="n"/>
     </row>
     <row r="735">
       <c r="A735" s="3" t="n">
@@ -13532,11 +13114,7 @@
       <c r="C735" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D735" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D735" s="4" t="n"/>
     </row>
     <row r="736">
       <c r="A736" s="5" t="n">
@@ -13550,11 +13128,7 @@
       <c r="C736" s="5" t="n">
         <v>2012</v>
       </c>
-      <c r="D736" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D736" s="6" t="n"/>
     </row>
     <row r="737">
       <c r="A737" s="3" t="n">
@@ -13568,11 +13142,7 @@
       <c r="C737" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D737" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D737" s="4" t="n"/>
     </row>
     <row r="738">
       <c r="A738" s="5" t="n">
@@ -13586,11 +13156,7 @@
       <c r="C738" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D738" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D738" s="6" t="n"/>
     </row>
     <row r="739">
       <c r="A739" s="3" t="n">
@@ -13604,11 +13170,7 @@
       <c r="C739" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D739" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D739" s="4" t="n"/>
     </row>
     <row r="740">
       <c r="A740" s="5" t="n">
@@ -13874,11 +13436,7 @@
       <c r="C754" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D754" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D754" s="6" t="n"/>
     </row>
     <row r="755">
       <c r="A755" s="3" t="n">
@@ -13892,11 +13450,7 @@
       <c r="C755" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D755" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D755" s="4" t="n"/>
     </row>
     <row r="756">
       <c r="A756" s="5" t="n">
@@ -14162,11 +13716,7 @@
       <c r="C770" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D770" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D770" s="6" t="n"/>
     </row>
     <row r="771">
       <c r="A771" s="3" t="n">
@@ -14180,11 +13730,7 @@
       <c r="C771" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D771" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D771" s="4" t="n"/>
     </row>
     <row r="772">
       <c r="A772" s="5" t="n">
@@ -14200,7 +13746,7 @@
       </c>
       <c r="D772" s="6" t="inlineStr">
         <is>
-          <t>bseindia.com/xml-data/corpfiling/AttachHis/24a0940c-fa5a-4e36-a404-9dab3637ea0c.pdf</t>
+          <t>https://bseindia.com/xml-data/corpfiling/AttachHis/24a0940c-fa5a-4e36-a404-9dab3637ea0c.pdf</t>
         </is>
       </c>
     </row>
@@ -14218,7 +13764,7 @@
       </c>
       <c r="D773" s="4" t="inlineStr">
         <is>
-          <t>bseindia.com/xml-data/corpfiling/AttachHis//ae413f27-7b30-4cdb-8f1b-8d82e5914e54.pdf</t>
+          <t>https://bseindia.com/xml-data/corpfiling/AttachHis//ae413f27-7b30-4cdb-8f1b-8d82e5914e54.pdf</t>
         </is>
       </c>
     </row>
@@ -14450,11 +13996,7 @@
       <c r="C786" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D786" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D786" s="6" t="n"/>
     </row>
     <row r="787">
       <c r="A787" s="3" t="n">
@@ -14468,11 +14010,7 @@
       <c r="C787" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D787" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D787" s="4" t="n"/>
     </row>
     <row r="788">
       <c r="A788" s="5" t="n">
@@ -14576,11 +14114,7 @@
       <c r="C793" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="D793" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D793" s="4" t="n"/>
     </row>
     <row r="794">
       <c r="A794" s="5" t="n">
@@ -14594,11 +14128,7 @@
       <c r="C794" s="5" t="n">
         <v>2018</v>
       </c>
-      <c r="D794" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D794" s="6" t="n"/>
     </row>
     <row r="795">
       <c r="A795" s="3" t="n">
@@ -14612,11 +14142,7 @@
       <c r="C795" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="D795" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D795" s="4" t="n"/>
     </row>
     <row r="796">
       <c r="A796" s="5" t="n">
@@ -14630,11 +14156,7 @@
       <c r="C796" s="5" t="n">
         <v>2016</v>
       </c>
-      <c r="D796" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D796" s="6" t="n"/>
     </row>
     <row r="797">
       <c r="A797" s="3" t="n">
@@ -14648,11 +14170,7 @@
       <c r="C797" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="D797" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D797" s="4" t="n"/>
     </row>
     <row r="798">
       <c r="A798" s="5" t="n">
@@ -14666,11 +14184,7 @@
       <c r="C798" s="5" t="n">
         <v>2014</v>
       </c>
-      <c r="D798" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D798" s="6" t="n"/>
     </row>
     <row r="799">
       <c r="A799" s="3" t="n">
@@ -14684,11 +14198,7 @@
       <c r="C799" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D799" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D799" s="4" t="n"/>
     </row>
     <row r="800">
       <c r="A800" s="5" t="n">
@@ -14702,11 +14212,7 @@
       <c r="C800" s="5" t="n">
         <v>2012</v>
       </c>
-      <c r="D800" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D800" s="6" t="n"/>
     </row>
     <row r="801">
       <c r="A801" s="3" t="n">
@@ -14720,11 +14226,7 @@
       <c r="C801" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D801" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D801" s="4" t="n"/>
     </row>
     <row r="802">
       <c r="A802" s="5" t="n">
@@ -14738,11 +14240,7 @@
       <c r="C802" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D802" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D802" s="6" t="n"/>
     </row>
     <row r="803">
       <c r="A803" s="3" t="n">
@@ -14756,11 +14254,7 @@
       <c r="C803" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D803" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D803" s="4" t="n"/>
     </row>
     <row r="804">
       <c r="A804" s="5" t="n">
@@ -14846,11 +14340,7 @@
       <c r="C808" s="5" t="n">
         <v>2020</v>
       </c>
-      <c r="D808" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D808" s="6" t="n"/>
     </row>
     <row r="809">
       <c r="A809" s="3" t="n">
@@ -14864,11 +14354,7 @@
       <c r="C809" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="D809" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D809" s="4" t="n"/>
     </row>
     <row r="810">
       <c r="A810" s="5" t="n">
@@ -14882,11 +14368,7 @@
       <c r="C810" s="5" t="n">
         <v>2018</v>
       </c>
-      <c r="D810" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D810" s="6" t="n"/>
     </row>
     <row r="811">
       <c r="A811" s="3" t="n">
@@ -14900,11 +14382,7 @@
       <c r="C811" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="D811" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D811" s="4" t="n"/>
     </row>
     <row r="812">
       <c r="A812" s="5" t="n">
@@ -14918,11 +14396,7 @@
       <c r="C812" s="5" t="n">
         <v>2016</v>
       </c>
-      <c r="D812" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D812" s="6" t="n"/>
     </row>
     <row r="813">
       <c r="A813" s="3" t="n">
@@ -14936,11 +14410,7 @@
       <c r="C813" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="D813" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D813" s="4" t="n"/>
     </row>
     <row r="814">
       <c r="A814" s="5" t="n">
@@ -14954,11 +14424,7 @@
       <c r="C814" s="5" t="n">
         <v>2014</v>
       </c>
-      <c r="D814" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D814" s="6" t="n"/>
     </row>
     <row r="815">
       <c r="A815" s="3" t="n">
@@ -14972,11 +14438,7 @@
       <c r="C815" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D815" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D815" s="4" t="n"/>
     </row>
     <row r="816">
       <c r="A816" s="5" t="n">
@@ -14990,11 +14452,7 @@
       <c r="C816" s="5" t="n">
         <v>2012</v>
       </c>
-      <c r="D816" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D816" s="6" t="n"/>
     </row>
     <row r="817">
       <c r="A817" s="3" t="n">
@@ -15008,11 +14466,7 @@
       <c r="C817" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D817" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D817" s="4" t="n"/>
     </row>
     <row r="818">
       <c r="A818" s="5" t="n">
@@ -15026,11 +14480,7 @@
       <c r="C818" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D818" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D818" s="6" t="n"/>
     </row>
     <row r="819">
       <c r="A819" s="3" t="n">
@@ -15044,11 +14494,7 @@
       <c r="C819" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D819" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D819" s="4" t="n"/>
     </row>
     <row r="820">
       <c r="A820" s="5" t="n">
@@ -15296,7 +14742,9 @@
       <c r="C833" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D833" s="4" t="n"/>
+      <c r="D833" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="834">
       <c r="A834" s="5" t="n">
@@ -15310,7 +14758,9 @@
       <c r="C834" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D834" s="6" t="n"/>
+      <c r="D834" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="835">
       <c r="A835" s="3" t="n">
@@ -15324,7 +14774,9 @@
       <c r="C835" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D835" s="4" t="n"/>
+      <c r="D835" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="836">
       <c r="A836" s="5" t="n">
@@ -15590,7 +15042,9 @@
       <c r="C850" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D850" s="6" t="n"/>
+      <c r="D850" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="851">
       <c r="A851" s="3" t="n">
@@ -15604,7 +15058,9 @@
       <c r="C851" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D851" s="4" t="n"/>
+      <c r="D851" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="852">
       <c r="A852" s="5" t="n">
@@ -15636,11 +15092,7 @@
       <c r="C853" s="3" t="n">
         <v>2023</v>
       </c>
-      <c r="D853" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D853" s="4" t="n"/>
     </row>
     <row r="854">
       <c r="A854" s="5" t="n">
@@ -15654,11 +15106,7 @@
       <c r="C854" s="5" t="n">
         <v>2022</v>
       </c>
-      <c r="D854" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D854" s="6" t="n"/>
     </row>
     <row r="855">
       <c r="A855" s="3" t="n">
@@ -15672,11 +15120,7 @@
       <c r="C855" s="3" t="n">
         <v>2021</v>
       </c>
-      <c r="D855" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D855" s="4" t="n"/>
     </row>
     <row r="856">
       <c r="A856" s="5" t="n">
@@ -15690,11 +15134,7 @@
       <c r="C856" s="5" t="n">
         <v>2020</v>
       </c>
-      <c r="D856" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D856" s="6" t="n"/>
     </row>
     <row r="857">
       <c r="A857" s="3" t="n">
@@ -15708,11 +15148,7 @@
       <c r="C857" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="D857" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D857" s="4" t="n"/>
     </row>
     <row r="858">
       <c r="A858" s="5" t="n">
@@ -15726,11 +15162,7 @@
       <c r="C858" s="5" t="n">
         <v>2018</v>
       </c>
-      <c r="D858" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D858" s="6" t="n"/>
     </row>
     <row r="859">
       <c r="A859" s="3" t="n">
@@ -15744,11 +15176,7 @@
       <c r="C859" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="D859" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D859" s="4" t="n"/>
     </row>
     <row r="860">
       <c r="A860" s="5" t="n">
@@ -15762,11 +15190,7 @@
       <c r="C860" s="5" t="n">
         <v>2016</v>
       </c>
-      <c r="D860" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D860" s="6" t="n"/>
     </row>
     <row r="861">
       <c r="A861" s="3" t="n">
@@ -15780,11 +15204,7 @@
       <c r="C861" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="D861" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D861" s="4" t="n"/>
     </row>
     <row r="862">
       <c r="A862" s="5" t="n">
@@ -15798,11 +15218,7 @@
       <c r="C862" s="5" t="n">
         <v>2014</v>
       </c>
-      <c r="D862" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D862" s="6" t="n"/>
     </row>
     <row r="863">
       <c r="A863" s="3" t="n">
@@ -15816,11 +15232,7 @@
       <c r="C863" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D863" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D863" s="4" t="n"/>
     </row>
     <row r="864">
       <c r="A864" s="5" t="n">
@@ -15834,11 +15246,7 @@
       <c r="C864" s="5" t="n">
         <v>2012</v>
       </c>
-      <c r="D864" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D864" s="6" t="n"/>
     </row>
     <row r="865">
       <c r="A865" s="3" t="n">
@@ -15852,11 +15260,7 @@
       <c r="C865" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D865" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D865" s="4" t="n"/>
     </row>
     <row r="866">
       <c r="A866" s="5" t="n">
@@ -15870,11 +15274,7 @@
       <c r="C866" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D866" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D866" s="6" t="n"/>
     </row>
     <row r="867">
       <c r="A867" s="3" t="n">
@@ -15888,11 +15288,7 @@
       <c r="C867" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D867" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D867" s="4" t="n"/>
     </row>
     <row r="868">
       <c r="A868" s="5" t="n">
@@ -16140,11 +15536,7 @@
       <c r="C881" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D881" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D881" s="4" t="n"/>
     </row>
     <row r="882">
       <c r="A882" s="5" t="n">
@@ -16158,11 +15550,7 @@
       <c r="C882" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D882" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D882" s="6" t="n"/>
     </row>
     <row r="883">
       <c r="A883" s="3" t="n">
@@ -16176,11 +15564,7 @@
       <c r="C883" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D883" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D883" s="4" t="n"/>
     </row>
     <row r="884">
       <c r="A884" s="5" t="n">
@@ -16446,11 +15830,7 @@
       <c r="C898" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D898" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D898" s="6" t="n"/>
     </row>
     <row r="899">
       <c r="A899" s="3" t="n">
@@ -16464,11 +15844,7 @@
       <c r="C899" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D899" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D899" s="4" t="n"/>
     </row>
     <row r="900">
       <c r="A900" s="5" t="n">
@@ -16502,7 +15878,7 @@
       </c>
       <c r="D901" s="4" t="inlineStr">
         <is>
-          <t>bseindia.com/xml-data/corpfiling/AttachHis//b9e0c871-3353-4ef4-855e-069bcfd848e1.pdf</t>
+          <t>https://bseindia.com/xml-data/corpfiling/AttachHis//b9e0c871-3353-4ef4-855e-069bcfd848e1.pdf</t>
         </is>
       </c>
     </row>
@@ -16520,7 +15896,7 @@
       </c>
       <c r="D902" s="6" t="inlineStr">
         <is>
-          <t>bseindia.com/bseplus/AnnualReport/500247/73932500247.pdf</t>
+          <t>https://bseindia.com/bseplus/AnnualReport/500247/73932500247.pdf</t>
         </is>
       </c>
     </row>
@@ -16538,7 +15914,7 @@
       </c>
       <c r="D903" s="4" t="inlineStr">
         <is>
-          <t>bseindia.com/bseplus/AnnualReport/500247/69160500247.pdf</t>
+          <t>https://bseindia.com/bseplus/AnnualReport/500247/69160500247.pdf</t>
         </is>
       </c>
     </row>
@@ -16610,7 +15986,7 @@
       </c>
       <c r="D907" s="4" t="inlineStr">
         <is>
-          <t>bseindia.com/bseplus/AnnualReport/500247/5002470317.pdf</t>
+          <t>https://bseindia.com/bseplus/AnnualReport/500247/5002470317.pdf</t>
         </is>
       </c>
     </row>
@@ -16628,7 +16004,7 @@
       </c>
       <c r="D908" s="6" t="inlineStr">
         <is>
-          <t>5002470316.pdf</t>
+          <t>https://5002470316.pdf</t>
         </is>
       </c>
     </row>
@@ -16646,7 +16022,7 @@
       </c>
       <c r="D909" s="4" t="inlineStr">
         <is>
-          <t>5002470315.pdf</t>
+          <t>https://5002470315.pdf</t>
         </is>
       </c>
     </row>
@@ -16682,7 +16058,7 @@
       </c>
       <c r="D911" s="4" t="inlineStr">
         <is>
-          <t>untitled</t>
+          <t>https://untitled</t>
         </is>
       </c>
     </row>
@@ -16700,7 +16076,7 @@
       </c>
       <c r="D912" s="6" t="inlineStr">
         <is>
-          <t>bseindia.com/bseplus/AnnualReport/500247/5002470312.pdf</t>
+          <t>https://bseindia.com/bseplus/AnnualReport/500247/5002470312.pdf</t>
         </is>
       </c>
     </row>
@@ -16718,7 +16094,7 @@
       </c>
       <c r="D913" s="4" t="inlineStr">
         <is>
-          <t>5002470311.pdf</t>
+          <t>https://5002470311.pdf</t>
         </is>
       </c>
     </row>
@@ -16734,11 +16110,7 @@
       <c r="C914" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D914" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D914" s="6" t="n"/>
     </row>
     <row r="915">
       <c r="A915" s="3" t="n">
@@ -16752,11 +16124,7 @@
       <c r="C915" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D915" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D915" s="4" t="n"/>
     </row>
     <row r="916">
       <c r="A916" s="5" t="n">
@@ -16878,11 +16246,7 @@
       <c r="C922" s="5" t="n">
         <v>2018</v>
       </c>
-      <c r="D922" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D922" s="6" t="n"/>
     </row>
     <row r="923">
       <c r="A923" s="3" t="n">
@@ -16896,11 +16260,7 @@
       <c r="C923" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="D923" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D923" s="4" t="n"/>
     </row>
     <row r="924">
       <c r="A924" s="5" t="n">
@@ -16914,11 +16274,7 @@
       <c r="C924" s="5" t="n">
         <v>2016</v>
       </c>
-      <c r="D924" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D924" s="6" t="n"/>
     </row>
     <row r="925">
       <c r="A925" s="3" t="n">
@@ -16932,11 +16288,7 @@
       <c r="C925" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="D925" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D925" s="4" t="n"/>
     </row>
     <row r="926">
       <c r="A926" s="5" t="n">
@@ -16950,11 +16302,7 @@
       <c r="C926" s="5" t="n">
         <v>2014</v>
       </c>
-      <c r="D926" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D926" s="6" t="n"/>
     </row>
     <row r="927">
       <c r="A927" s="3" t="n">
@@ -16968,11 +16316,7 @@
       <c r="C927" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D927" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D927" s="4" t="n"/>
     </row>
     <row r="928">
       <c r="A928" s="5" t="n">
@@ -16986,11 +16330,7 @@
       <c r="C928" s="5" t="n">
         <v>2012</v>
       </c>
-      <c r="D928" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D928" s="6" t="n"/>
     </row>
     <row r="929">
       <c r="A929" s="3" t="n">
@@ -17004,11 +16344,7 @@
       <c r="C929" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D929" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D929" s="4" t="n"/>
     </row>
     <row r="930">
       <c r="A930" s="5" t="n">
@@ -17022,11 +16358,7 @@
       <c r="C930" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D930" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D930" s="6" t="n"/>
     </row>
     <row r="931">
       <c r="A931" s="3" t="n">
@@ -17040,11 +16372,7 @@
       <c r="C931" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D931" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D931" s="4" t="n"/>
     </row>
     <row r="932">
       <c r="A932" s="5" t="n">
@@ -17130,11 +16458,7 @@
       <c r="C936" s="5" t="n">
         <v>2020</v>
       </c>
-      <c r="D936" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D936" s="6" t="n"/>
     </row>
     <row r="937">
       <c r="A937" s="3" t="n">
@@ -17148,11 +16472,7 @@
       <c r="C937" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="D937" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D937" s="4" t="n"/>
     </row>
     <row r="938">
       <c r="A938" s="5" t="n">
@@ -17166,11 +16486,7 @@
       <c r="C938" s="5" t="n">
         <v>2018</v>
       </c>
-      <c r="D938" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D938" s="6" t="n"/>
     </row>
     <row r="939">
       <c r="A939" s="3" t="n">
@@ -17184,11 +16500,7 @@
       <c r="C939" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="D939" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D939" s="4" t="n"/>
     </row>
     <row r="940">
       <c r="A940" s="5" t="n">
@@ -17202,11 +16514,7 @@
       <c r="C940" s="5" t="n">
         <v>2016</v>
       </c>
-      <c r="D940" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D940" s="6" t="n"/>
     </row>
     <row r="941">
       <c r="A941" s="3" t="n">
@@ -17220,11 +16528,7 @@
       <c r="C941" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="D941" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D941" s="4" t="n"/>
     </row>
     <row r="942">
       <c r="A942" s="5" t="n">
@@ -17238,11 +16542,7 @@
       <c r="C942" s="5" t="n">
         <v>2014</v>
       </c>
-      <c r="D942" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D942" s="6" t="n"/>
     </row>
     <row r="943">
       <c r="A943" s="3" t="n">
@@ -17256,11 +16556,7 @@
       <c r="C943" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D943" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D943" s="4" t="n"/>
     </row>
     <row r="944">
       <c r="A944" s="5" t="n">
@@ -17274,11 +16570,7 @@
       <c r="C944" s="5" t="n">
         <v>2012</v>
       </c>
-      <c r="D944" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D944" s="6" t="n"/>
     </row>
     <row r="945">
       <c r="A945" s="3" t="n">
@@ -17292,11 +16584,7 @@
       <c r="C945" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D945" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D945" s="4" t="n"/>
     </row>
     <row r="946">
       <c r="A946" s="5" t="n">
@@ -17310,11 +16598,7 @@
       <c r="C946" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D946" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D946" s="6" t="n"/>
     </row>
     <row r="947">
       <c r="A947" s="3" t="n">
@@ -17328,11 +16612,7 @@
       <c r="C947" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D947" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D947" s="4" t="n"/>
     </row>
     <row r="948">
       <c r="A948" s="5" t="n">
@@ -17598,11 +16878,7 @@
       <c r="C962" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D962" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D962" s="6" t="n"/>
     </row>
     <row r="963">
       <c r="A963" s="3" t="n">
@@ -17616,11 +16892,7 @@
       <c r="C963" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D963" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D963" s="4" t="n"/>
     </row>
     <row r="964">
       <c r="A964" s="5" t="n">
@@ -17778,11 +17050,7 @@
       <c r="C972" s="5" t="n">
         <v>2016</v>
       </c>
-      <c r="D972" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D972" s="6" t="n"/>
     </row>
     <row r="973">
       <c r="A973" s="3" t="n">
@@ -17796,11 +17064,7 @@
       <c r="C973" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="D973" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D973" s="4" t="n"/>
     </row>
     <row r="974">
       <c r="A974" s="5" t="n">
@@ -17814,11 +17078,7 @@
       <c r="C974" s="5" t="n">
         <v>2014</v>
       </c>
-      <c r="D974" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D974" s="6" t="n"/>
     </row>
     <row r="975">
       <c r="A975" s="3" t="n">
@@ -17832,11 +17092,7 @@
       <c r="C975" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D975" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D975" s="4" t="n"/>
     </row>
     <row r="976">
       <c r="A976" s="5" t="n">
@@ -17850,11 +17106,7 @@
       <c r="C976" s="5" t="n">
         <v>2012</v>
       </c>
-      <c r="D976" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D976" s="6" t="n"/>
     </row>
     <row r="977">
       <c r="A977" s="3" t="n">
@@ -17868,11 +17120,7 @@
       <c r="C977" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D977" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D977" s="4" t="n"/>
     </row>
     <row r="978">
       <c r="A978" s="5" t="n">
@@ -17886,11 +17134,7 @@
       <c r="C978" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D978" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D978" s="6" t="n"/>
     </row>
     <row r="979">
       <c r="A979" s="3" t="n">
@@ -17904,11 +17148,7 @@
       <c r="C979" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D979" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D979" s="4" t="n"/>
     </row>
     <row r="980">
       <c r="A980" s="5" t="n">
@@ -18174,11 +17414,7 @@
       <c r="C994" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D994" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D994" s="6" t="n"/>
     </row>
     <row r="995">
       <c r="A995" s="3" t="n">
@@ -18192,11 +17428,7 @@
       <c r="C995" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D995" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D995" s="4" t="n"/>
     </row>
     <row r="996">
       <c r="A996" s="5" t="n">
@@ -18462,11 +17694,7 @@
       <c r="C1010" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1010" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1010" s="6" t="n"/>
     </row>
     <row r="1011">
       <c r="A1011" s="3" t="n">
@@ -18480,11 +17708,7 @@
       <c r="C1011" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1011" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1011" s="4" t="n"/>
     </row>
     <row r="1012">
       <c r="A1012" s="5" t="n">
@@ -18750,11 +17974,7 @@
       <c r="C1026" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1026" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1026" s="6" t="n"/>
     </row>
     <row r="1027">
       <c r="A1027" s="3" t="n">
@@ -18768,11 +17988,7 @@
       <c r="C1027" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1027" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1027" s="4" t="n"/>
     </row>
     <row r="1028">
       <c r="A1028" s="5" t="n">
@@ -19038,11 +18254,7 @@
       <c r="C1042" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1042" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1042" s="6" t="n"/>
     </row>
     <row r="1043">
       <c r="A1043" s="3" t="n">
@@ -19056,11 +18268,7 @@
       <c r="C1043" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1043" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1043" s="4" t="n"/>
     </row>
     <row r="1044">
       <c r="A1044" s="5" t="n">
@@ -19092,7 +18300,9 @@
       <c r="C1045" s="3" t="n">
         <v>2023</v>
       </c>
-      <c r="D1045" s="4" t="n"/>
+      <c r="D1045" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1046">
       <c r="A1046" s="5" t="n">
@@ -19610,11 +18820,7 @@
       <c r="C1074" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1074" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1074" s="6" t="n"/>
     </row>
     <row r="1075">
       <c r="A1075" s="3" t="n">
@@ -19628,11 +18834,7 @@
       <c r="C1075" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1075" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1075" s="4" t="n"/>
     </row>
     <row r="1076">
       <c r="A1076" s="5" t="n">
@@ -19898,11 +19100,7 @@
       <c r="C1090" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1090" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1090" s="6" t="n"/>
     </row>
     <row r="1091">
       <c r="A1091" s="3" t="n">
@@ -19916,11 +19114,7 @@
       <c r="C1091" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1091" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1091" s="4" t="n"/>
     </row>
     <row r="1092">
       <c r="A1092" s="5" t="n">
@@ -20168,11 +19362,7 @@
       <c r="C1105" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1105" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1105" s="4" t="n"/>
     </row>
     <row r="1106">
       <c r="A1106" s="5" t="n">
@@ -20186,11 +19376,7 @@
       <c r="C1106" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1106" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1106" s="6" t="n"/>
     </row>
     <row r="1107">
       <c r="A1107" s="3" t="n">
@@ -20204,11 +19390,7 @@
       <c r="C1107" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1107" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1107" s="4" t="n"/>
     </row>
     <row r="1108">
       <c r="A1108" s="5" t="n">
@@ -20474,11 +19656,7 @@
       <c r="C1122" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1122" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1122" s="6" t="n"/>
     </row>
     <row r="1123">
       <c r="A1123" s="3" t="n">
@@ -20492,11 +19670,7 @@
       <c r="C1123" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1123" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1123" s="4" t="n"/>
     </row>
     <row r="1124">
       <c r="A1124" s="5" t="n">
@@ -20744,11 +19918,7 @@
       <c r="C1137" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1137" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1137" s="4" t="n"/>
     </row>
     <row r="1138">
       <c r="A1138" s="5" t="n">
@@ -20762,11 +19932,7 @@
       <c r="C1138" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1138" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1138" s="6" t="n"/>
     </row>
     <row r="1139">
       <c r="A1139" s="3" t="n">
@@ -20780,11 +19946,7 @@
       <c r="C1139" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1139" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1139" s="4" t="n"/>
     </row>
     <row r="1140">
       <c r="A1140" s="5" t="n">
@@ -21050,11 +20212,7 @@
       <c r="C1154" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1154" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1154" s="6" t="n"/>
     </row>
     <row r="1155">
       <c r="A1155" s="3" t="n">
@@ -21068,11 +20226,7 @@
       <c r="C1155" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1155" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1155" s="4" t="n"/>
     </row>
     <row r="1156">
       <c r="A1156" s="5" t="n">
@@ -21338,11 +20492,7 @@
       <c r="C1170" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1170" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1170" s="6" t="n"/>
     </row>
     <row r="1171">
       <c r="A1171" s="3" t="n">
@@ -21356,11 +20506,7 @@
       <c r="C1171" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1171" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1171" s="4" t="n"/>
     </row>
     <row r="1172">
       <c r="A1172" s="5" t="n">
@@ -21608,11 +20754,7 @@
       <c r="C1185" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1185" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1185" s="4" t="n"/>
     </row>
     <row r="1186">
       <c r="A1186" s="5" t="n">
@@ -21626,11 +20768,7 @@
       <c r="C1186" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1186" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1186" s="6" t="n"/>
     </row>
     <row r="1187">
       <c r="A1187" s="3" t="n">
@@ -21644,11 +20782,7 @@
       <c r="C1187" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1187" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1187" s="4" t="n"/>
     </row>
     <row r="1188">
       <c r="A1188" s="5" t="n">
@@ -21896,11 +21030,7 @@
       <c r="C1201" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1201" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1201" s="4" t="n"/>
     </row>
     <row r="1202">
       <c r="A1202" s="5" t="n">
@@ -21914,11 +21044,7 @@
       <c r="C1202" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1202" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1202" s="6" t="n"/>
     </row>
     <row r="1203">
       <c r="A1203" s="3" t="n">
@@ -21932,11 +21058,7 @@
       <c r="C1203" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1203" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1203" s="4" t="n"/>
     </row>
     <row r="1204">
       <c r="A1204" s="5" t="n">
@@ -22076,11 +21198,7 @@
       <c r="C1211" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="D1211" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1211" s="4" t="n"/>
     </row>
     <row r="1212">
       <c r="A1212" s="5" t="n">
@@ -22094,11 +21212,7 @@
       <c r="C1212" s="5" t="n">
         <v>2016</v>
       </c>
-      <c r="D1212" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1212" s="6" t="n"/>
     </row>
     <row r="1213">
       <c r="A1213" s="3" t="n">
@@ -22112,11 +21226,7 @@
       <c r="C1213" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="D1213" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1213" s="4" t="n"/>
     </row>
     <row r="1214">
       <c r="A1214" s="5" t="n">
@@ -22130,11 +21240,7 @@
       <c r="C1214" s="5" t="n">
         <v>2014</v>
       </c>
-      <c r="D1214" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1214" s="6" t="n"/>
     </row>
     <row r="1215">
       <c r="A1215" s="3" t="n">
@@ -22148,11 +21254,7 @@
       <c r="C1215" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D1215" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1215" s="4" t="n"/>
     </row>
     <row r="1216">
       <c r="A1216" s="5" t="n">
@@ -22166,11 +21268,7 @@
       <c r="C1216" s="5" t="n">
         <v>2012</v>
       </c>
-      <c r="D1216" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1216" s="6" t="n"/>
     </row>
     <row r="1217">
       <c r="A1217" s="3" t="n">
@@ -22184,11 +21282,7 @@
       <c r="C1217" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1217" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1217" s="4" t="n"/>
     </row>
     <row r="1218">
       <c r="A1218" s="5" t="n">
@@ -22202,11 +21296,7 @@
       <c r="C1218" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1218" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1218" s="6" t="n"/>
     </row>
     <row r="1219">
       <c r="A1219" s="3" t="n">
@@ -22220,11 +21310,7 @@
       <c r="C1219" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1219" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1219" s="4" t="n"/>
     </row>
     <row r="1220">
       <c r="A1220" s="5" t="n">
@@ -22508,11 +21594,7 @@
       <c r="C1235" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1235" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1235" s="4" t="n"/>
     </row>
     <row r="1236">
       <c r="A1236" s="5" t="n">
@@ -22760,11 +21842,7 @@
       <c r="C1249" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1249" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1249" s="4" t="n"/>
     </row>
     <row r="1250">
       <c r="A1250" s="5" t="n">
@@ -22778,11 +21856,7 @@
       <c r="C1250" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1250" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1250" s="6" t="n"/>
     </row>
     <row r="1251">
       <c r="A1251" s="3" t="n">
@@ -22796,11 +21870,7 @@
       <c r="C1251" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1251" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1251" s="4" t="n"/>
     </row>
     <row r="1252">
       <c r="A1252" s="5" t="n">
@@ -23048,11 +22118,7 @@
       <c r="C1265" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1265" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1265" s="4" t="n"/>
     </row>
     <row r="1266">
       <c r="A1266" s="5" t="n">
@@ -23066,11 +22132,7 @@
       <c r="C1266" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1266" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1266" s="6" t="n"/>
     </row>
     <row r="1267">
       <c r="A1267" s="3" t="n">
@@ -23084,11 +22146,7 @@
       <c r="C1267" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1267" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1267" s="4" t="n"/>
     </row>
     <row r="1268">
       <c r="A1268" s="5" t="n">
@@ -23354,11 +22412,7 @@
       <c r="C1282" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1282" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1282" s="6" t="n"/>
     </row>
     <row r="1283">
       <c r="A1283" s="3" t="n">
@@ -23372,11 +22426,7 @@
       <c r="C1283" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1283" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1283" s="4" t="n"/>
     </row>
     <row r="1284">
       <c r="A1284" s="5" t="n">
@@ -23624,7 +22674,9 @@
       <c r="C1297" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1297" s="4" t="n"/>
+      <c r="D1297" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1298">
       <c r="A1298" s="5" t="n">
@@ -23638,7 +22690,9 @@
       <c r="C1298" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1298" s="6" t="n"/>
+      <c r="D1298" s="6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1299">
       <c r="A1299" s="3" t="n">
@@ -23652,7 +22706,9 @@
       <c r="C1299" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1299" s="4" t="n"/>
+      <c r="D1299" s="4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="1300">
       <c r="A1300" s="5" t="n">
@@ -23918,11 +22974,7 @@
       <c r="C1314" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1314" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1314" s="6" t="n"/>
     </row>
     <row r="1315">
       <c r="A1315" s="3" t="n">
@@ -23936,11 +22988,7 @@
       <c r="C1315" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1315" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1315" s="4" t="n"/>
     </row>
     <row r="1316">
       <c r="A1316" s="5" t="n">
@@ -24206,11 +23254,7 @@
       <c r="C1330" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1330" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1330" s="6" t="n"/>
     </row>
     <row r="1331">
       <c r="A1331" s="3" t="n">
@@ -24224,11 +23268,7 @@
       <c r="C1331" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1331" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1331" s="4" t="n"/>
     </row>
     <row r="1332">
       <c r="A1332" s="5" t="n">
@@ -24494,11 +23534,7 @@
       <c r="C1346" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1346" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1346" s="6" t="n"/>
     </row>
     <row r="1347">
       <c r="A1347" s="3" t="n">
@@ -24512,11 +23548,7 @@
       <c r="C1347" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1347" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1347" s="4" t="n"/>
     </row>
     <row r="1348">
       <c r="A1348" s="5" t="n">
@@ -24782,11 +23814,7 @@
       <c r="C1362" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1362" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1362" s="6" t="n"/>
     </row>
     <row r="1363">
       <c r="A1363" s="3" t="n">
@@ -24800,11 +23828,7 @@
       <c r="C1363" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1363" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1363" s="4" t="n"/>
     </row>
     <row r="1364">
       <c r="A1364" s="5" t="n">
@@ -25070,11 +24094,7 @@
       <c r="C1378" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1378" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1378" s="6" t="n"/>
     </row>
     <row r="1379">
       <c r="A1379" s="3" t="n">
@@ -25088,11 +24108,7 @@
       <c r="C1379" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1379" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1379" s="4" t="n"/>
     </row>
     <row r="1380">
       <c r="A1380" s="5" t="n">
@@ -25322,11 +24338,7 @@
       <c r="C1392" s="5" t="n">
         <v>2012</v>
       </c>
-      <c r="D1392" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1392" s="6" t="n"/>
     </row>
     <row r="1393">
       <c r="A1393" s="3" t="n">
@@ -25340,11 +24352,7 @@
       <c r="C1393" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1393" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1393" s="4" t="n"/>
     </row>
     <row r="1394">
       <c r="A1394" s="5" t="n">
@@ -25358,11 +24366,7 @@
       <c r="C1394" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1394" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1394" s="6" t="n"/>
     </row>
     <row r="1395">
       <c r="A1395" s="3" t="n">
@@ -25376,11 +24380,7 @@
       <c r="C1395" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1395" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1395" s="4" t="n"/>
     </row>
     <row r="1396">
       <c r="A1396" s="5" t="n">
@@ -25628,11 +24628,7 @@
       <c r="C1409" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1409" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1409" s="4" t="n"/>
     </row>
     <row r="1410">
       <c r="A1410" s="5" t="n">
@@ -25646,11 +24642,7 @@
       <c r="C1410" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1410" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1410" s="6" t="n"/>
     </row>
     <row r="1411">
       <c r="A1411" s="3" t="n">
@@ -25664,11 +24656,7 @@
       <c r="C1411" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1411" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1411" s="4" t="n"/>
     </row>
     <row r="1412">
       <c r="A1412" s="5" t="n">
@@ -25934,11 +24922,7 @@
       <c r="C1426" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1426" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1426" s="6" t="n"/>
     </row>
     <row r="1427">
       <c r="A1427" s="3" t="n">
@@ -25952,11 +24936,7 @@
       <c r="C1427" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1427" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1427" s="4" t="n"/>
     </row>
     <row r="1428">
       <c r="A1428" s="5" t="n">
@@ -26222,11 +25202,7 @@
       <c r="C1442" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1442" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1442" s="6" t="n"/>
     </row>
     <row r="1443">
       <c r="A1443" s="3" t="n">
@@ -26240,11 +25216,7 @@
       <c r="C1443" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1443" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1443" s="4" t="n"/>
     </row>
     <row r="1444">
       <c r="A1444" s="5" t="n">
@@ -26510,11 +25482,7 @@
       <c r="C1458" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1458" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1458" s="6" t="n"/>
     </row>
     <row r="1459">
       <c r="A1459" s="3" t="n">
@@ -26528,11 +25496,7 @@
       <c r="C1459" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1459" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1459" s="4" t="n"/>
     </row>
     <row r="1460">
       <c r="A1460" s="5" t="n">
@@ -26780,11 +25744,7 @@
       <c r="C1473" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1473" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1473" s="4" t="n"/>
     </row>
     <row r="1474">
       <c r="A1474" s="5" t="n">
@@ -26798,11 +25758,7 @@
       <c r="C1474" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1474" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1474" s="6" t="n"/>
     </row>
     <row r="1475">
       <c r="A1475" s="3" t="n">
@@ -26816,11 +25772,7 @@
       <c r="C1475" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1475" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1475" s="4" t="n"/>
     </row>
     <row r="1476">
       <c r="A1476" s="5" t="n">
@@ -27086,11 +26038,7 @@
       <c r="C1490" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1490" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1490" s="6" t="n"/>
     </row>
     <row r="1491">
       <c r="A1491" s="3" t="n">
@@ -27104,11 +26052,7 @@
       <c r="C1491" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1491" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1491" s="4" t="n"/>
     </row>
     <row r="1492">
       <c r="A1492" s="5" t="n">
@@ -27356,11 +26300,7 @@
       <c r="C1505" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1505" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1505" s="4" t="n"/>
     </row>
     <row r="1506">
       <c r="A1506" s="5" t="n">
@@ -27374,11 +26314,7 @@
       <c r="C1506" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1506" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1506" s="6" t="n"/>
     </row>
     <row r="1507">
       <c r="A1507" s="3" t="n">
@@ -27392,11 +26328,7 @@
       <c r="C1507" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1507" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1507" s="4" t="n"/>
     </row>
     <row r="1508">
       <c r="A1508" s="5" t="n">
@@ -27410,11 +26342,7 @@
       <c r="C1508" s="5" t="n">
         <v>2024</v>
       </c>
-      <c r="D1508" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1508" s="6" t="n"/>
     </row>
     <row r="1509">
       <c r="A1509" s="3" t="n">
@@ -27572,11 +26500,7 @@
       <c r="C1517" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="D1517" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1517" s="4" t="n"/>
     </row>
     <row r="1518">
       <c r="A1518" s="5" t="n">
@@ -27590,11 +26514,7 @@
       <c r="C1518" s="5" t="n">
         <v>2014</v>
       </c>
-      <c r="D1518" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1518" s="6" t="n"/>
     </row>
     <row r="1519">
       <c r="A1519" s="3" t="n">
@@ -27608,11 +26528,7 @@
       <c r="C1519" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D1519" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1519" s="4" t="n"/>
     </row>
     <row r="1520">
       <c r="A1520" s="5" t="n">
@@ -27626,11 +26542,7 @@
       <c r="C1520" s="5" t="n">
         <v>2012</v>
       </c>
-      <c r="D1520" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1520" s="6" t="n"/>
     </row>
     <row r="1521">
       <c r="A1521" s="3" t="n">
@@ -27644,11 +26556,7 @@
       <c r="C1521" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1521" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1521" s="4" t="n"/>
     </row>
     <row r="1522">
       <c r="A1522" s="5" t="n">
@@ -27662,11 +26570,7 @@
       <c r="C1522" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1522" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1522" s="6" t="n"/>
     </row>
     <row r="1523">
       <c r="A1523" s="3" t="n">
@@ -27680,11 +26584,7 @@
       <c r="C1523" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1523" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1523" s="4" t="n"/>
     </row>
     <row r="1524">
       <c r="A1524" s="5" t="n">
@@ -27950,11 +26850,7 @@
       <c r="C1538" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1538" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1538" s="6" t="n"/>
     </row>
     <row r="1539">
       <c r="A1539" s="3" t="n">
@@ -27968,11 +26864,7 @@
       <c r="C1539" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1539" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1539" s="4" t="n"/>
     </row>
     <row r="1540">
       <c r="A1540" s="5" t="n">
@@ -28238,11 +27130,7 @@
       <c r="C1554" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1554" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1554" s="6" t="n"/>
     </row>
     <row r="1555">
       <c r="A1555" s="3" t="n">
@@ -28256,11 +27144,7 @@
       <c r="C1555" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1555" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1555" s="4" t="n"/>
     </row>
     <row r="1556">
       <c r="A1556" s="5" t="n">
@@ -28328,11 +27212,7 @@
       <c r="C1559" s="3" t="n">
         <v>2021</v>
       </c>
-      <c r="D1559" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1559" s="4" t="n"/>
     </row>
     <row r="1560">
       <c r="A1560" s="5" t="n">
@@ -28346,11 +27226,7 @@
       <c r="C1560" s="5" t="n">
         <v>2020</v>
       </c>
-      <c r="D1560" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1560" s="6" t="n"/>
     </row>
     <row r="1561">
       <c r="A1561" s="3" t="n">
@@ -28364,11 +27240,7 @@
       <c r="C1561" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="D1561" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1561" s="4" t="n"/>
     </row>
     <row r="1562">
       <c r="A1562" s="5" t="n">
@@ -28382,11 +27254,7 @@
       <c r="C1562" s="5" t="n">
         <v>2018</v>
       </c>
-      <c r="D1562" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1562" s="6" t="n"/>
     </row>
     <row r="1563">
       <c r="A1563" s="3" t="n">
@@ -28400,11 +27268,7 @@
       <c r="C1563" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="D1563" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1563" s="4" t="n"/>
     </row>
     <row r="1564">
       <c r="A1564" s="5" t="n">
@@ -28418,11 +27282,7 @@
       <c r="C1564" s="5" t="n">
         <v>2016</v>
       </c>
-      <c r="D1564" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1564" s="6" t="n"/>
     </row>
     <row r="1565">
       <c r="A1565" s="3" t="n">
@@ -28436,11 +27296,7 @@
       <c r="C1565" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="D1565" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1565" s="4" t="n"/>
     </row>
     <row r="1566">
       <c r="A1566" s="5" t="n">
@@ -28454,11 +27310,7 @@
       <c r="C1566" s="5" t="n">
         <v>2014</v>
       </c>
-      <c r="D1566" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1566" s="6" t="n"/>
     </row>
     <row r="1567">
       <c r="A1567" s="3" t="n">
@@ -28472,11 +27324,7 @@
       <c r="C1567" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="D1567" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1567" s="4" t="n"/>
     </row>
     <row r="1568">
       <c r="A1568" s="5" t="n">
@@ -28490,11 +27338,7 @@
       <c r="C1568" s="5" t="n">
         <v>2012</v>
       </c>
-      <c r="D1568" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1568" s="6" t="n"/>
     </row>
     <row r="1569">
       <c r="A1569" s="3" t="n">
@@ -28508,11 +27352,7 @@
       <c r="C1569" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="D1569" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1569" s="4" t="n"/>
     </row>
     <row r="1570">
       <c r="A1570" s="5" t="n">
@@ -28526,11 +27366,7 @@
       <c r="C1570" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1570" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1570" s="6" t="n"/>
     </row>
     <row r="1571">
       <c r="A1571" s="3" t="n">
@@ -28544,11 +27380,7 @@
       <c r="C1571" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1571" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1571" s="4" t="n"/>
     </row>
     <row r="1572">
       <c r="A1572" s="5" t="n">
@@ -28814,11 +27646,7 @@
       <c r="C1586" s="5" t="n">
         <v>2010</v>
       </c>
-      <c r="D1586" s="6" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1586" s="6" t="n"/>
     </row>
     <row r="1587">
       <c r="A1587" s="3" t="n">
@@ -28832,11 +27660,7 @@
       <c r="C1587" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="D1587" s="4" t="inlineStr">
-        <is>
-          <t>Null</t>
-        </is>
-      </c>
+      <c r="D1587" s="4" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:D2"/>

</xml_diff>